<commit_message>
Automatiza 42 arquivo(s) de processos no backend
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG BACKLIGHT MOD 4.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG BACKLIGHT MOD 4.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -25,10 +25,6 @@
       <name val="Carlito"/>
       <color rgb="FF17313A"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Carlito"/>
-      <sz val="8"/>
     </font>
   </fonts>
   <fills count="2">
@@ -341,7 +337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -944,6 +940,566 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Quadro do Corpo LE</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>22</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>001766</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Quadro do Corpo LD</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>22</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>001767</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Quadro Testeira</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="n">
+        <v>44</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>001768</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Testeira</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>22</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>001769</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Canaleta Testeira</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>22</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>001770</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Corpo Central</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>22</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>001771</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Trava Corpo Central</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>22</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>001772</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Estrutura Lat Esq</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="n">
+        <v>22</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>001773</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Estrutura Lat Dir</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>22</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>001774</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Cruzeta</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>44</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>001775</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Parachoque</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" t="n">
+        <v>44</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>001776</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Chapa do rodizio corpo lateral</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" t="n">
+        <v>44</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>001777</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Bdj Maior Lateral</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>8</v>
+      </c>
+      <c r="E34" t="n">
+        <v>176</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>001778</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Arame na Bdj Maior Lat</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>8</v>
+      </c>
+      <c r="E35" t="n">
+        <v>176</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>001779</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Bdj Menor Lateral</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" t="n">
+        <v>44</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>001780</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Arame na Bdj Menor Lat</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" t="n">
+        <v>44</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>001781</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Bdj Central</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>4</v>
+      </c>
+      <c r="E38" t="n">
+        <v>88</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>001782</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Arame na Bdj Central</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>4</v>
+      </c>
+      <c r="E39" t="n">
+        <v>88</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>001783</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Tubo Curvo Arte Direita</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>22</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>001784</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>PG BACKLIGHT MOD 4</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Tubo Curvo Arte Esquerda</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" t="n">
+        <v>22</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>001785</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>